<commit_message>
Update _b_fetchModelData; stop tracking build/dist artifacts and add .gitignore
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,27 +418,27 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>144</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>('Analysis Messages', 'Analysis Options - Active Degrees of Freedom', 'Analysis Options - Analysis Model for Nonlinear Hinges', 'Analysis Options - Automatic Mesh Settings for Floors', 'Analysis Options - Automatic Rectangular Mesh Options for Walls', 'Analysis Options - Cracking Analysis Options', 'Analysis Options - Design and Response Recovery Options', 'Analysis Options - SAPFire Options', 'Area Assignments - Auto Edge Constraints', 'Area Assignments - Floor Auto Mesh Options', 'Area Assignments - Insertion Point', 'Area Assignments - Local Axes', 'Area Assignments - Section Properties', 'Area Assignments - Summary', 'Area Load Assignments - Uniform', 'Area Section Property Definitions - Summary', 'Assembled Joint Masses', 'Base Reactions', 'Beam Bays', 'Beam Object Connectivity', 'Composite Beam Additional Sections With Studs', 'Composite Beam Design Envelope', 'Composite Beam Design Envelope - AISC 360-16', 'Composite Beam Design Overwrites - AISC 360-16', 'Composite Beam Design Preferences - AISC 360-16', 'Composite Beam Design Summary - AISC 360-16', 'Composite Column Design Preferences - AISC 360-16', 'Concrete Frame Design Preferences - ACI 318-14', 'Concrete Slab Design Overwrites - Punching Shear - General', 'Concrete Slab Design Preferences - ACI 318-14', 'Deck Property Definitions', 'Design Forces - Beams', 'Diaphragm Definitions', 'Diaphragm Forces', 'Dimension Line Object Geometry', 'Element Forces - Area Shells', 'Element Forces - Beams', 'Element Joint Forces - Frame', 'Element Joint Forces - Shells', 'Element Strains - Area Shells', 'Element Stresses - Area Shells', 'Floor Bays', 'Floor Object Connectivity', 'Frame Assignments - End Length Offsets', 'Frame Assignments - Frame Auto Mesh Options', 'Frame Assignments - Insertion Point', 'Frame Assignments - Local Axes', 'Frame Assignments - Output Stations', 'Frame Assignments - Releases and Partial Fixity', 'Frame Assignments - Section Properties', 'Frame Assignments - Summary', 'Frame Loads Assignments - Open Structure Wind Parameters', 'Frame Section Property Definitions - Concrete Beam Reinforcing', 'Frame Section Property Definitions - Concrete Column Reinforcing', 'Frame Section Property Definitions - Concrete Rectangular', 'Frame Section Property Definitions - Section Designer', 'Frame Section Property Definitions - Steel Angle', 'Frame Section Property Definitions - Steel I/Wide Flange', 'Frame Section Property Definitions - Summary', 'Functions - Response Spectrum - User Defined', 'Functions - Time History - User Defined', 'Grid Definitions - General', 'Grid Definitions - Grid Lines', 'Group Assignments', 'Group Definitions', 'Joint Assignments - Restraints', 'Joint Assignments - Summary', 'Joint Design Reactions', 'Joint Displacements', 'Joint Displacements (Including Internal Mesh Joints)', 'Joint Drifts', 'Joint Reactions', 'Link Property Definitions - Linear', 'Link Property Definitions - Summary', 'Load Case Definitions - Linear Static', 'Load Case Definitions - Summary', 'Load Combination Definitions', 'Load Pattern Definitions', 'Mass Source Definition', 'Mass Summary by Group', 'Mass Summary by Story', 'Material List by Object Type', 'Material List by Section Property', 'Material List by Story', 'Material Properties - Acceptance Criteria', 'Material Properties - Basic Mechanical Properties', 'Material Properties - Coldformed Data', 'Material Properties - Concrete Data', 'Material Properties - Damping Parameters', 'Material Properties - General', 'Material Properties - Hysteresis Parameters - Concrete', 'Material Properties - Rebar Data', 'Material Properties - Steel Data', 'Material Properties - Tendon Data', 'Material Properties - User Stress-Strain Curves', 'Miscellaneous Options', 'Modal Case Definitions - Eigen', 'Modal Direction Factors', 'Modal Load Participation Ratios', 'Modal Participating Mass Ratios', 'Modal Participation Factors', 'Modal Periods And Frequencies', 'Null Area Bays', 'Null Area Object Connectivity', 'Objects and Elements - Areas', 'Objects and Elements - Frames', 'Objects and Elements - Joints', 'Options - Colors - Display', 'Options - Colors - Output', 'Panel Zone Property Definitions', 'Pier Label Definitions', 'Point Bays', 'Point Object Connectivity', 'Preferences - Graphics', 'Preferences - Tolerance', 'Program Control', 'Project Information', 'Reinforcing Bar Sizes', 'Section Designer Shapes - Concrete Rectangle', 'Section Designer Shapes - Reinforcing - Line Bar', 'Section Designer Shapes - Steel I-Section', 'Shear Wall Design Preferences - ACI 318-14', 'Shear Wall Design Preferences - ACI 530-11 Masonry', 'Shear Wall Design Preferences - AISC 360-22 Composite', 'Shell Uniform Load Sets', 'Slab Property Definitions', 'Spandrel Label Definitions', 'Steel Beam Deflection Envelope - AISC 360-16', 'Steel Beam Envelope - AISC 360-16', 'Steel Design Load Combination Data', 'Steel Frame Design Overwrites - AISC 360-16', 'Steel Frame Design Preferences - AISC 360-16', 'Steel Frame Design Summary - AISC 360-16', 'Steel Joist Design Preferences - SJI-2010', 'Story Definitions', 'Story Drifts', 'Story Forces', 'Story Max Over Avg Displacements', 'Story Max Over Avg Drifts', 'Story Stiffness', 'Tendon Section Properties', 'Tower and Base Story Definitions', 'Tributary Area and LLRF', 'Wall Property Definitions - Specified')</t>
+          <t>('Analysis Options - Active Degrees of Freedom', 'Analysis Options - Analysis Model for Nonlinear Hinges', 'Analysis Options - Automatic Mesh Settings for Floors', 'Analysis Options - Automatic Rectangular Mesh Options for Walls', 'Analysis Options - Cracking Analysis Options', 'Analysis Options - Design and Response Recovery Options', 'Analysis Options - SAPFire Options', 'Area Assignments - Auto Edge Constraints', 'Area Assignments - Floor Auto Mesh Options', 'Area Assignments - Insertion Point', 'Area Assignments - Local Axes', 'Area Assignments - Section Properties', 'Area Assignments - Summary', 'Area Load Assignments - Uniform', 'Area Section Property Definitions - Summary', 'Beam Bays', 'Beam Object Connectivity', 'Column Bays', 'Column Object Connectivity', 'Composite Beam Additional Sections With Studs', 'Composite Beam Design Overwrites - AISC 360-16', 'Composite Beam Design Preferences - AISC 360-16', 'Composite Column Design Preferences - AISC 360-16', 'Concrete Frame Design Preferences - ACI 318-14', 'Concrete Slab Design Overwrites - Punching Shear - General', 'Concrete Slab Design Preferences - ACI 318-14', 'Deck Property Definitions', 'Diaphragm Definitions', 'Dimension Line Object Geometry', 'Floor Bays', 'Floor Object Connectivity', 'Frame Assignments - End Length Offsets', 'Frame Assignments - Frame Auto Mesh Options', 'Frame Assignments - Insertion Point', 'Frame Assignments - Local Axes', 'Frame Assignments - Output Stations', 'Frame Assignments - Releases and Partial Fixity', 'Frame Assignments - Section Properties', 'Frame Assignments - Summary', 'Frame Loads Assignments - Open Structure Wind Parameters', 'Frame Section Property Definitions - Concrete Beam Reinforcing', 'Frame Section Property Definitions - Concrete Column Reinforcing', 'Frame Section Property Definitions - Concrete Rectangular', 'Frame Section Property Definitions - Section Designer', 'Frame Section Property Definitions - Steel Angle', 'Frame Section Property Definitions - Steel I/Wide Flange', 'Frame Section Property Definitions - Summary', 'Functions - Response Spectrum - User Defined', 'Functions - Time History - User Defined', 'Grid Definitions - General', 'Grid Definitions - Grid Lines', 'Group Assignments', 'Group Definitions', 'Joint Assignments - Restraints', 'Joint Assignments - Summary', 'Joint Loads Assignments - Force', 'Link Property Definitions - Linear', 'Link Property Definitions - Summary', 'Load Case Definitions - Linear Static', 'Load Case Definitions - Summary', 'Load Combination Definitions', 'Load Pattern Definitions', 'Mass Source Definition', 'Material List by Object Type', 'Material List by Section Property', 'Material List by Story', 'Material Properties - Acceptance Criteria', 'Material Properties - Basic Mechanical Properties', 'Material Properties - Coldformed Data', 'Material Properties - Concrete Data', 'Material Properties - Damping Parameters', 'Material Properties - General', 'Material Properties - Hysteresis Parameters - Concrete', 'Material Properties - Rebar Data', 'Material Properties - Steel Data', 'Material Properties - Tendon Data', 'Material Properties - User Stress-Strain Curves', 'Miscellaneous Options', 'Modal Case Definitions - Eigen', 'Null Area Bays', 'Null Area Object Connectivity', 'Null Line Bays', 'Null Line Object Connectivity', 'Options - Colors - Display', 'Options - Colors - Output', 'Panel Zone Property Definitions', 'Pier Label Definitions', 'Point Bays', 'Point Object Connectivity', 'Preferences - Graphics', 'Preferences - Tolerance', 'Program Control', 'Project Information', 'Reinforcing Bar Sizes', 'Section Designer Shapes - Concrete Rectangle', 'Section Designer Shapes - Reinforcing - Line Bar', 'Section Designer Shapes - Steel I-Section', 'Shear Wall Design Preferences - ACI 318-14', 'Shear Wall Design Preferences - ACI 530-11 Masonry', 'Shear Wall Design Preferences - AISC 360-22 Composite', 'Shell Uniform Load Sets', 'Slab Property Definitions', 'Spandrel Label Definitions', 'Steel Design Load Combination Data', 'Steel Frame Design Overwrites - AISC 360-16', 'Steel Frame Design Preferences - AISC 360-16', 'Steel Joist Design Preferences - SJI-2010', 'Story Definitions', 'Tendon Section Properties', 'Tower and Base Story Definitions', 'Wall Property Definitions - Specified')</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>('Analysis Messages', 'Analysis Options - Active Degrees of Freedom', 'Analysis Options - Analysis Model for Nonlinear Hinges', 'Analysis Options - Automatic Mesh Settings for Floors', 'Analysis Options - Automatic Rectangular Mesh Options for Walls', 'Analysis Options - Cracking Analysis Options', 'Analysis Options - Design and Response Recovery Options', 'Analysis Options - SAPFire Options', 'Area Assignments - Auto Edge Constraints', 'Area Assignments - Floor Auto Mesh Options', 'Area Assignments - Insertion Point', 'Area Assignments - Local Axes', 'Area Assignments - Section Properties', 'Area Assignments - Summary', 'Area Load Assignments - Uniform', 'Area Section Property Definitions - Summary', 'Assembled Joint Masses', 'Base Reactions', 'Beam Bays', 'Beam Object Connectivity', 'Composite Beam Additional Sections With Studs', 'Composite Beam Design Envelope', 'Composite Beam Design Envelope - AISC 360-16', 'Composite Beam Design Overwrites - AISC 360-16', 'Composite Beam Design Preferences - AISC 360-16', 'Composite Beam Design Summary - AISC 360-16', 'Composite Column Design Preferences - AISC 360-16', 'Concrete Frame Design Preferences - ACI 318-14', 'Concrete Slab Design Overwrites - Punching Shear - General', 'Concrete Slab Design Preferences - ACI 318-14', 'Deck Property Definitions', 'Design Forces - Beams', 'Diaphragm Definitions', 'Diaphragm Forces', 'Dimension Line Object Geometry', 'Element Forces - Area Shells', 'Element Forces - Beams', 'Element Joint Forces - Frame', 'Element Joint Forces - Shells', 'Element Strains - Area Shells', 'Element Stresses - Area Shells', 'Floor Bays', 'Floor Object Connectivity', 'Frame Assignments - End Length Offsets', 'Frame Assignments - Frame Auto Mesh Options', 'Frame Assignments - Insertion Point', 'Frame Assignments - Local Axes', 'Frame Assignments - Output Stations', 'Frame Assignments - Releases and Partial Fixity', 'Frame Assignments - Section Properties', 'Frame Assignments - Summary', 'Frame Loads Assignments - Open Structure Wind Parameters', 'Frame Section Property Definitions - Concrete Beam Reinforcing', 'Frame Section Property Definitions - Concrete Column Reinforcing', 'Frame Section Property Definitions - Concrete Rectangular', 'Frame Section Property Definitions - Section Designer', 'Frame Section Property Definitions - Steel Angle', 'Frame Section Property Definitions - Steel I/Wide Flange', 'Frame Section Property Definitions - Summary', 'Functions - Response Spectrum - User Defined', 'Functions - Time History - User Defined', 'Grid Definitions - General', 'Grid Definitions - Grid Lines', 'Group Assignments', 'Group Definitions', 'Joint Assignments - Restraints', 'Joint Assignments - Summary', 'Joint Design Reactions', 'Joint Displacements', 'Joint Displacements (Including Internal Mesh Joints)', 'Joint Drifts', 'Joint Reactions', 'Link Property Definitions - Linear', 'Link Property Definitions - Summary', 'Load Case Definitions - Linear Static', 'Load Case Definitions - Summary', 'Load Combination Definitions', 'Load Pattern Definitions', 'Mass Source Definition', 'Mass Summary by Group', 'Mass Summary by Story', 'Material List by Object Type', 'Material List by Section Property', 'Material List by Story', 'Material Properties - Acceptance Criteria', 'Material Properties - Basic Mechanical Properties', 'Material Properties - Coldformed Data', 'Material Properties - Concrete Data', 'Material Properties - Damping Parameters', 'Material Properties - General', 'Material Properties - Hysteresis Parameters - Concrete', 'Material Properties - Rebar Data', 'Material Properties - Steel Data', 'Material Properties - Tendon Data', 'Material Properties - User Stress-Strain Curves', 'Miscellaneous Options', 'Modal Case Definitions - Eigen', 'Modal Direction Factors', 'Modal Load Participation Ratios', 'Modal Participating Mass Ratios', 'Modal Participation Factors', 'Modal Periods And Frequencies', 'Null Area Bays', 'Null Area Object Connectivity', 'Objects and Elements - Areas', 'Objects and Elements - Frames', 'Objects and Elements - Joints', 'Options - Colors - Display', 'Options - Colors - Output', 'Panel Zone Property Definitions', 'Pier Label Definitions', 'Point Bays', 'Point Object Connectivity', 'Preferences - Graphics', 'Preferences - Tolerance', 'Program Control', 'Project Information', 'Reinforcing Bar Sizes', 'Section Designer Shapes - Concrete Rectangle', 'Section Designer Shapes - Reinforcing - Line Bar', 'Section Designer Shapes - Steel I-Section', 'Shear Wall Design Preferences - ACI 318-14', 'Shear Wall Design Preferences - ACI 530-11 Masonry', 'Shear Wall Design Preferences - AISC 360-22 Composite', 'Shell Uniform Load Sets', 'Slab Property Definitions', 'Spandrel Label Definitions', 'Steel Beam Deflection Envelope - AISC 360-16', 'Steel Beam Envelope - AISC 360-16', 'Steel Design Load Combination Data', 'Steel Frame Design Overwrites - AISC 360-16', 'Steel Frame Design Preferences - AISC 360-16', 'Steel Frame Design Summary - AISC 360-16', 'Steel Joist Design Preferences - SJI-2010', 'Story Definitions', 'Story Drifts', 'Story Forces', 'Story Max Over Avg Displacements', 'Story Max Over Avg Drifts', 'Story Stiffness', 'Tendon Section Properties', 'Tower and Base Story Definitions', 'Tributary Area and LLRF', 'Wall Property Definitions - Specified')</t>
+          <t>('Analysis Options - Active Degrees of Freedom', 'Analysis Options - Analysis Model for Nonlinear Hinges', 'Analysis Options - Automatic Mesh Settings for Floors', 'Analysis Options - Automatic Rectangular Mesh Options for Walls', 'Analysis Options - Cracking Analysis Options', 'Analysis Options - Design and Response Recovery Options', 'Analysis Options - SAPFire Options', 'Area Assignments - Auto Edge Constraints', 'Area Assignments - Floor Auto Mesh Options', 'Area Assignments - Insertion Point', 'Area Assignments - Local Axes', 'Area Assignments - Section Properties', 'Area Assignments - Summary', 'Area Load Assignments - Uniform', 'Area Section Property Definitions - Summary', 'Beam Bays', 'Beam Object Connectivity', 'Column Bays', 'Column Object Connectivity', 'Composite Beam Additional Sections With Studs', 'Composite Beam Design Overwrites - AISC 360-16', 'Composite Beam Design Preferences - AISC 360-16', 'Composite Column Design Preferences - AISC 360-16', 'Concrete Frame Design Preferences - ACI 318-14', 'Concrete Slab Design Overwrites - Punching Shear - General', 'Concrete Slab Design Preferences - ACI 318-14', 'Deck Property Definitions', 'Diaphragm Definitions', 'Dimension Line Object Geometry', 'Floor Bays', 'Floor Object Connectivity', 'Frame Assignments - End Length Offsets', 'Frame Assignments - Frame Auto Mesh Options', 'Frame Assignments - Insertion Point', 'Frame Assignments - Local Axes', 'Frame Assignments - Output Stations', 'Frame Assignments - Releases and Partial Fixity', 'Frame Assignments - Section Properties', 'Frame Assignments - Summary', 'Frame Loads Assignments - Open Structure Wind Parameters', 'Frame Section Property Definitions - Concrete Beam Reinforcing', 'Frame Section Property Definitions - Concrete Column Reinforcing', 'Frame Section Property Definitions - Concrete Rectangular', 'Frame Section Property Definitions - Section Designer', 'Frame Section Property Definitions - Steel Angle', 'Frame Section Property Definitions - Steel I/Wide Flange', 'Frame Section Property Definitions - Summary', 'Functions - Response Spectrum - User Defined', 'Functions - Time History - User Defined', 'Grid Definitions - General', 'Grid Definitions - Grid Lines', 'Group Assignments', 'Group Definitions', 'Joint Assignments - Restraints', 'Joint Assignments - Summary', 'Joint Loads Assignments - Force', 'Link Property Definitions - Linear', 'Link Property Definitions - Summary', 'Load Case Definitions - Linear Static', 'Load Case Definitions - Summary', 'Load Combination Definitions', 'Load Pattern Definitions', 'Mass Source Definition', 'Material List by Object Type', 'Material List by Section Property', 'Material List by Story', 'Material Properties - Acceptance Criteria', 'Material Properties - Basic Mechanical Properties', 'Material Properties - Coldformed Data', 'Material Properties - Concrete Data', 'Material Properties - Damping Parameters', 'Material Properties - General', 'Material Properties - Hysteresis Parameters - Concrete', 'Material Properties - Rebar Data', 'Material Properties - Steel Data', 'Material Properties - Tendon Data', 'Material Properties - User Stress-Strain Curves', 'Miscellaneous Options', 'Modal Case Definitions - Eigen', 'Null Area Bays', 'Null Area Object Connectivity', 'Null Line Bays', 'Null Line Object Connectivity', 'Options - Colors - Display', 'Options - Colors - Output', 'Panel Zone Property Definitions', 'Pier Label Definitions', 'Point Bays', 'Point Object Connectivity', 'Preferences - Graphics', 'Preferences - Tolerance', 'Program Control', 'Project Information', 'Reinforcing Bar Sizes', 'Section Designer Shapes - Concrete Rectangle', 'Section Designer Shapes - Reinforcing - Line Bar', 'Section Designer Shapes - Steel I-Section', 'Shear Wall Design Preferences - ACI 318-14', 'Shear Wall Design Preferences - ACI 530-11 Masonry', 'Shear Wall Design Preferences - AISC 360-22 Composite', 'Shell Uniform Load Sets', 'Slab Property Definitions', 'Spandrel Label Definitions', 'Steel Design Load Combination Data', 'Steel Frame Design Overwrites - AISC 360-16', 'Steel Frame Design Preferences - AISC 360-16', 'Steel Joist Design Preferences - SJI-2010', 'Story Definitions', 'Tendon Section Properties', 'Tower and Base Story Definitions', 'Wall Property Definitions - Specified')</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>(0, 2, 2, 2, 2, 2, 3, 2, 2, 2, 2, 2, 2, 0, 2, 0, 0, 0, 0, 2, 3, 0, 0, 3, 3, 0, 3, 3, 3, 3, 2, 0, 2, 0, 2, 0, 0, 0, 0, 0, 0, 0, 2, 2, 2, 2, 2, 2, 2, 2, 0, 2, 2, 2, 2, 2, 2, 2, 0, 2, 2, 2, 2, 2, 2, 2, 0, 0, 0, 0, 0, 0, 2, 0, 2, 0, 2, 2, 2, 0, 0, 0, 0, 0, 2, 2, 2, 2, 2, 2, 2, 2, 2, 2, 2, 3, 2, 0, 0, 0, 0, 0, 0, 2, 0, 0, 0, 3, 3, 2, 3, 0, 2, 3, 3, 3, 3, 2, 2, 2, 2, 3, 3, 3, 2, 2, 3, 0, 0, 3, 3, 3, 0, 3, 1, 0, 0, 0, 0, 0, 2, 1, 0, 2)</t>
+          <t>(2, 2, 2, 2, 2, 3, 2, 2, 2, 2, 2, 2, 0, 2, 0, 0, 2, 0, 2, 3, 3, 3, 3, 3, 3, 3, 2, 2, 2, 0, 2, 2, 2, 2, 2, 2, 2, 2, 0, 2, 2, 2, 2, 2, 2, 2, 0, 2, 2, 2, 2, 2, 2, 2, 0, 2, 2, 0, 2, 0, 2, 2, 2, 0, 0, 0, 2, 2, 2, 2, 2, 2, 2, 2, 2, 2, 2, 3, 2, 0, 2, 0, 2, 3, 3, 2, 3, 0, 2, 3, 3, 3, 3, 2, 2, 2, 2, 3, 3, 3, 2, 2, 3, 3, 3, 3, 3, 1, 2, 1, 2)</t>
         </is>
       </c>
     </row>

</xml_diff>